<commit_message>
corrections sur la plateforme
</commit_message>
<xml_diff>
--- a/output/QAQC_rapport.xlsx
+++ b/output/QAQC_rapport.xlsx
@@ -1861,7 +1861,7 @@
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>cm_secteur_emploi</t>
+          <t>cm_revenu</t>
         </is>
       </c>
       <c r="B2" s="10" t="n">
@@ -1879,7 +1879,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>cm_statut_emploi</t>
+          <t>cm_secteur_emploi</t>
         </is>
       </c>
       <c r="B3" s="10" t="n">
@@ -1897,7 +1897,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>cm_situation_matrimoniale</t>
+          <t>cm_statut_emploi</t>
         </is>
       </c>
       <c r="B4" s="10" t="n">
@@ -1915,7 +1915,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>cm_revenu</t>
+          <t>cm_situation_matrimoniale</t>
         </is>
       </c>
       <c r="B5" s="10" t="n">
@@ -2005,7 +2005,7 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>montant_evacuation_tranche</t>
+          <t>frequence_paiement</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
@@ -2023,7 +2023,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>frequence_paiement</t>
+          <t>montant_evacuation_tranche</t>
         </is>
       </c>
       <c r="B11" s="10" t="n">
@@ -2149,7 +2149,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>service_evacuation_payant</t>
+          <t>service_alternatif_raison</t>
         </is>
       </c>
       <c r="B18" s="10" t="n">
@@ -2167,7 +2167,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>service_alternatif_raison</t>
+          <t>service_alternatif_type</t>
         </is>
       </c>
       <c r="B19" s="10" t="n">
@@ -2185,7 +2185,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>service_alternatif_type</t>
+          <t>service_evacuation_payant</t>
         </is>
       </c>
       <c r="B20" s="10" t="n">
@@ -2383,7 +2383,7 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>satisfaction_benne</t>
+          <t>responsable_evacuation</t>
         </is>
       </c>
       <c r="B31" s="11" t="n">
@@ -2401,7 +2401,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>frequence_benne</t>
+          <t>satisfaction_benne</t>
         </is>
       </c>
       <c r="B32" s="11" t="n">
@@ -2419,7 +2419,7 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>responsable_evacuation</t>
+          <t>benne_point_nettoyage</t>
         </is>
       </c>
       <c r="B33" s="11" t="n">
@@ -2437,7 +2437,7 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>benne_point_nettoyage</t>
+          <t>distance_point_collecte</t>
         </is>
       </c>
       <c r="B34" s="11" t="n">
@@ -2455,7 +2455,7 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>benne_heure_convient</t>
+          <t>frequence_benne</t>
         </is>
       </c>
       <c r="B35" s="11" t="n">
@@ -2473,7 +2473,7 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>distance_point_collecte</t>
+          <t>benne_heure_convient</t>
         </is>
       </c>
       <c r="B36" s="11" t="n">
@@ -2671,7 +2671,7 @@
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>commune_libelle</t>
+          <t>commune_code</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
@@ -2689,7 +2689,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>commune_code</t>
+          <t>commune_libelle</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
@@ -2743,7 +2743,7 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>nat__v12</t>
+          <t>region</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
@@ -2761,7 +2761,7 @@
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>nb_adultes_H</t>
+          <t>quartier</t>
         </is>
       </c>
       <c r="B52" s="7" t="n">
@@ -2779,7 +2779,7 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>place_publique</t>
+          <t>nb_enfants_0_4</t>
         </is>
       </c>
       <c r="B53" s="8" t="n">
@@ -2797,7 +2797,7 @@
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>set_setal</t>
+          <t>zone</t>
         </is>
       </c>
       <c r="B54" s="7" t="n">
@@ -2815,7 +2815,7 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>statut_occupation</t>
+          <t>src__v3</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
@@ -2833,7 +2833,7 @@
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>nb_nuisibles</t>
+          <t>src__v4</t>
         </is>
       </c>
       <c r="B56" s="7" t="n">
@@ -2851,7 +2851,7 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>type_habitat</t>
+          <t>src__v5</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
@@ -2869,7 +2869,7 @@
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>nuisible__v29</t>
+          <t>cm_sexe</t>
         </is>
       </c>
       <c r="B58" s="7" t="n">
@@ -2887,7 +2887,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>nuisible__v28</t>
+          <t>repondant_statut</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
@@ -2905,7 +2905,7 @@
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>nuisible__v27</t>
+          <t>repondant_est_cm</t>
         </is>
       </c>
       <c r="B60" s="7" t="n">
@@ -2923,7 +2923,7 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>nuisible__v26</t>
+          <t>repondant_sexe</t>
         </is>
       </c>
       <c r="B61" s="8" t="n">
@@ -2941,7 +2941,7 @@
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>nuisible__v25</t>
+          <t>cm_alpha_arabe</t>
         </is>
       </c>
       <c r="B62" s="7" t="n">
@@ -2959,7 +2959,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>nuisible__v24</t>
+          <t>cm_alpha_anglais</t>
         </is>
       </c>
       <c r="B63" s="8" t="n">
@@ -2977,7 +2977,7 @@
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>nuisible__v23</t>
+          <t>cm_alpha_francais</t>
         </is>
       </c>
       <c r="B64" s="7" t="n">
@@ -2995,7 +2995,7 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>proxy_niveau_vie</t>
+          <t>cm_type_enseignement</t>
         </is>
       </c>
       <c r="B65" s="8" t="n">
@@ -3031,7 +3031,7 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>repondant_sexe</t>
+          <t>type_habitat</t>
         </is>
       </c>
       <c r="B67" s="8" t="n">
@@ -3049,7 +3049,7 @@
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>depots_sauvages_observes</t>
+          <t>proxy_niveau_vie</t>
         </is>
       </c>
       <c r="B68" s="7" t="n">
@@ -3067,7 +3067,7 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>eaux_usees_rue_freq</t>
+          <t>statut_occupation</t>
         </is>
       </c>
       <c r="B69" s="8" t="n">
@@ -3085,7 +3085,7 @@
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
         <is>
-          <t>nb_adultes_F</t>
+          <t>nb_enfants_5_15</t>
         </is>
       </c>
       <c r="B70" s="7" t="n">
@@ -3103,7 +3103,7 @@
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>nb_enfants_5_15</t>
+          <t>nb_adultes_H</t>
         </is>
       </c>
       <c r="B71" s="8" t="n">
@@ -3121,7 +3121,7 @@
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
         <is>
-          <t>nat__v13</t>
+          <t>nb_adultes_F</t>
         </is>
       </c>
       <c r="B72" s="7" t="n">
@@ -3139,7 +3139,7 @@
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>maladie__v34</t>
+          <t>au_moins_un_traitement</t>
         </is>
       </c>
       <c r="B73" s="8" t="n">
@@ -3157,7 +3157,7 @@
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
         <is>
-          <t>nb_types_maladies_menage</t>
+          <t>proportion_traitee</t>
         </is>
       </c>
       <c r="B74" s="7" t="n">
@@ -3175,7 +3175,7 @@
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>aucune_maladie</t>
+          <t>mode_stockage</t>
         </is>
       </c>
       <c r="B75" s="8" t="n">
@@ -3193,7 +3193,7 @@
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
         <is>
-          <t>nb_maladies</t>
+          <t>stockage_couvert</t>
         </is>
       </c>
       <c r="B76" s="7" t="n">
@@ -3211,7 +3211,7 @@
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>maladies_liste</t>
+          <t>capacite_stockage_suffisante</t>
         </is>
       </c>
       <c r="B77" s="8" t="n">
@@ -3229,7 +3229,7 @@
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
         <is>
-          <t>maladie__v38</t>
+          <t>place_stockage</t>
         </is>
       </c>
       <c r="B78" s="7" t="n">
@@ -3247,7 +3247,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>maladie__v37</t>
+          <t>revente_dechets</t>
         </is>
       </c>
       <c r="B79" s="8" t="n">
@@ -3265,7 +3265,7 @@
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
         <is>
-          <t>maladie__v36</t>
+          <t>tri_avant_evacuation</t>
         </is>
       </c>
       <c r="B80" s="7" t="n">
@@ -3283,7 +3283,7 @@
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>maladie__v35</t>
+          <t>nat__v12</t>
         </is>
       </c>
       <c r="B81" s="8" t="n">
@@ -3301,7 +3301,7 @@
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
         <is>
-          <t>maladie__v33</t>
+          <t>nat__v13</t>
         </is>
       </c>
       <c r="B82" s="7" t="n">
@@ -3319,7 +3319,7 @@
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
         <is>
-          <t>nb_enfants_0_4</t>
+          <t>nat__v14</t>
         </is>
       </c>
       <c r="B83" s="8" t="n">
@@ -3337,7 +3337,7 @@
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
         <is>
-          <t>maladie__v32</t>
+          <t>nat__v15</t>
         </is>
       </c>
       <c r="B84" s="7" t="n">
@@ -3355,7 +3355,7 @@
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>maladie__v31</t>
+          <t>nat__v16</t>
         </is>
       </c>
       <c r="B85" s="8" t="n">
@@ -3373,7 +3373,7 @@
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
         <is>
-          <t>maladie__v30</t>
+          <t>nat__v17</t>
         </is>
       </c>
       <c r="B86" s="7" t="n">
@@ -3391,7 +3391,7 @@
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>quartier</t>
+          <t>natures_liste</t>
         </is>
       </c>
       <c r="B87" s="8" t="n">
@@ -3409,7 +3409,7 @@
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>nb_natures</t>
         </is>
       </c>
       <c r="B88" s="7" t="n">
@@ -3427,7 +3427,7 @@
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>campagne_sensibilisation</t>
+          <t>nat__v11</t>
         </is>
       </c>
       <c r="B89" s="8" t="n">
@@ -3445,7 +3445,7 @@
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
         <is>
-          <t>connait_UCG</t>
+          <t>nat__v10</t>
         </is>
       </c>
       <c r="B90" s="7" t="n">
@@ -3463,7 +3463,7 @@
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>zone</t>
+          <t>nat__v9</t>
         </is>
       </c>
       <c r="B91" s="8" t="n">
@@ -3481,7 +3481,7 @@
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
         <is>
-          <t>dep_sauvages_rue_freq</t>
+          <t>nat__v8</t>
         </is>
       </c>
       <c r="B92" s="7" t="n">
@@ -3499,7 +3499,7 @@
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>acces_depotoire_normalise</t>
+          <t>nb_sources</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
@@ -3517,7 +3517,7 @@
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
         <is>
-          <t>repondant_statut</t>
+          <t>sources_liste</t>
         </is>
       </c>
       <c r="B94" s="7" t="n">
@@ -3535,7 +3535,7 @@
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>capacite_stockage_suffisante</t>
+          <t>src__v7</t>
         </is>
       </c>
       <c r="B95" s="8" t="n">
@@ -3553,7 +3553,7 @@
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
         <is>
-          <t>nb_sources</t>
+          <t>src__v6</t>
         </is>
       </c>
       <c r="B96" s="7" t="n">
@@ -3571,7 +3571,7 @@
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>nat__v8</t>
+          <t>cm_est_alphabetise</t>
         </is>
       </c>
       <c r="B97" s="8" t="n">
@@ -3589,7 +3589,7 @@
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
         <is>
-          <t>nat__v9</t>
+          <t>cm_alpha_autre_etrangere</t>
         </is>
       </c>
       <c r="B98" s="7" t="n">
@@ -3607,7 +3607,7 @@
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>proportion_traitee</t>
+          <t>cm_alpha_lng_nationale</t>
         </is>
       </c>
       <c r="B99" s="8" t="n">
@@ -3625,7 +3625,7 @@
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
         <is>
-          <t>nat__v10</t>
+          <t>src__v1</t>
         </is>
       </c>
       <c r="B100" s="7" t="n">
@@ -3643,7 +3643,7 @@
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>nat__v11</t>
+          <t>src__v2</t>
         </is>
       </c>
       <c r="B101" s="8" t="n">
@@ -3661,7 +3661,7 @@
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
         <is>
-          <t>revente_dechets</t>
+          <t>existence_bacs_quartier</t>
         </is>
       </c>
       <c r="B102" s="7" t="n">
@@ -3679,7 +3679,7 @@
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>tri_avant_evacuation</t>
+          <t>montant_mensuel_evacuation_fcfa</t>
         </is>
       </c>
       <c r="B103" s="8" t="n">
@@ -3697,7 +3697,7 @@
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
         <is>
-          <t>place_stockage</t>
+          <t>a_service_alternatif</t>
         </is>
       </c>
       <c r="B104" s="7" t="n">
@@ -3715,7 +3715,7 @@
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>au_moins_un_traitement</t>
+          <t>nuisible__v27</t>
         </is>
       </c>
       <c r="B105" s="8" t="n">
@@ -3733,7 +3733,7 @@
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
         <is>
-          <t>stockage_couvert</t>
+          <t>nuisible__v26</t>
         </is>
       </c>
       <c r="B106" s="7" t="n">
@@ -3751,7 +3751,7 @@
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t>mode_stockage</t>
+          <t>nuisible__v25</t>
         </is>
       </c>
       <c r="B107" s="8" t="n">
@@ -3769,7 +3769,7 @@
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
         <is>
-          <t>nb_natures</t>
+          <t>nuisible__v24</t>
         </is>
       </c>
       <c r="B108" s="7" t="n">
@@ -3787,7 +3787,7 @@
     <row r="109">
       <c r="A109" s="8" t="inlineStr">
         <is>
-          <t>natures_liste</t>
+          <t>nuisible__v23</t>
         </is>
       </c>
       <c r="B109" s="8" t="n">
@@ -3805,7 +3805,7 @@
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
         <is>
-          <t>nat__v17</t>
+          <t>dep_sauvages_rue_freq</t>
         </is>
       </c>
       <c r="B110" s="7" t="n">
@@ -3823,7 +3823,7 @@
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>nat__v16</t>
+          <t>eaux_usees_rue_freq</t>
         </is>
       </c>
       <c r="B111" s="8" t="n">
@@ -3841,7 +3841,7 @@
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
         <is>
-          <t>nat__v15</t>
+          <t>depots_sauvages_observes</t>
         </is>
       </c>
       <c r="B112" s="7" t="n">
@@ -3859,7 +3859,7 @@
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t>nat__v14</t>
+          <t>corbeilles_rue_presentes</t>
         </is>
       </c>
       <c r="B113" s="8" t="n">
@@ -3877,7 +3877,7 @@
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
         <is>
-          <t>sources_liste</t>
+          <t>acces_depotoire_normalise</t>
         </is>
       </c>
       <c r="B114" s="7" t="n">
@@ -3895,7 +3895,7 @@
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>src__v7</t>
+          <t>duree_quartier</t>
         </is>
       </c>
       <c r="B115" s="8" t="n">
@@ -3913,7 +3913,7 @@
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
         <is>
-          <t>repondant_est_cm</t>
+          <t>place_publique</t>
         </is>
       </c>
       <c r="B116" s="7" t="n">
@@ -3931,7 +3931,7 @@
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>cm_alpha_arabe</t>
+          <t>nuisible__v28</t>
         </is>
       </c>
       <c r="B117" s="8" t="n">
@@ -3949,7 +3949,7 @@
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
         <is>
-          <t>corbeilles_rue_presentes</t>
+          <t>set_setal</t>
         </is>
       </c>
       <c r="B118" s="7" t="n">
@@ -3967,7 +3967,7 @@
     <row r="119">
       <c r="A119" s="8" t="inlineStr">
         <is>
-          <t>cm_sexe</t>
+          <t>nuisible__v29</t>
         </is>
       </c>
       <c r="B119" s="8" t="n">
@@ -3985,7 +3985,7 @@
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
         <is>
-          <t>cm_type_enseignement</t>
+          <t>nb_nuisibles</t>
         </is>
       </c>
       <c r="B120" s="7" t="n">
@@ -4003,7 +4003,7 @@
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t>existence_bacs_quartier</t>
+          <t>campagne_sensibilisation</t>
         </is>
       </c>
       <c r="B121" s="8" t="n">
@@ -4021,7 +4021,7 @@
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
         <is>
-          <t>duree_quartier</t>
+          <t>connait_UCG</t>
         </is>
       </c>
       <c r="B122" s="7" t="n">
@@ -4039,7 +4039,7 @@
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>montant_mensuel_evacuation_fcfa</t>
+          <t>maladie__v30</t>
         </is>
       </c>
       <c r="B123" s="8" t="n">
@@ -4057,7 +4057,7 @@
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
         <is>
-          <t>cm_alpha_francais</t>
+          <t>maladie__v31</t>
         </is>
       </c>
       <c r="B124" s="7" t="n">
@@ -4075,7 +4075,7 @@
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>cm_alpha_anglais</t>
+          <t>maladie__v32</t>
         </is>
       </c>
       <c r="B125" s="8" t="n">
@@ -4093,7 +4093,7 @@
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
         <is>
-          <t>a_service_alternatif</t>
+          <t>maladie__v33</t>
         </is>
       </c>
       <c r="B126" s="7" t="n">
@@ -4111,7 +4111,7 @@
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t>src__v6</t>
+          <t>maladie__v34</t>
         </is>
       </c>
       <c r="B127" s="8" t="n">
@@ -4129,7 +4129,7 @@
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
         <is>
-          <t>cm_alpha_lng_nationale</t>
+          <t>maladie__v35</t>
         </is>
       </c>
       <c r="B128" s="7" t="n">
@@ -4147,7 +4147,7 @@
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t>cm_alpha_autre_etrangere</t>
+          <t>maladie__v36</t>
         </is>
       </c>
       <c r="B129" s="8" t="n">
@@ -4165,7 +4165,7 @@
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
         <is>
-          <t>cm_est_alphabetise</t>
+          <t>maladie__v37</t>
         </is>
       </c>
       <c r="B130" s="7" t="n">
@@ -4183,7 +4183,7 @@
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t>src__v1</t>
+          <t>maladie__v38</t>
         </is>
       </c>
       <c r="B131" s="8" t="n">
@@ -4201,7 +4201,7 @@
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
         <is>
-          <t>src__v2</t>
+          <t>maladies_liste</t>
         </is>
       </c>
       <c r="B132" s="7" t="n">
@@ -4219,7 +4219,7 @@
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t>src__v3</t>
+          <t>nb_maladies</t>
         </is>
       </c>
       <c r="B133" s="8" t="n">
@@ -4237,7 +4237,7 @@
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
-          <t>src__v4</t>
+          <t>aucune_maladie</t>
         </is>
       </c>
       <c r="B134" s="7" t="n">
@@ -4255,7 +4255,7 @@
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t>src__v5</t>
+          <t>nb_types_maladies_menage</t>
         </is>
       </c>
       <c r="B135" s="8" t="n">

</xml_diff>